<commit_message>
refactor(advisor): 落地恒等题号,移除 MP_TO_PY 翻译层
将 advisor 全链路内部题号迁到「与小程序一致」,gsyg_selectFinal 不再翻译。

- advisor_port.js:SCORE_CSV/ABILITY_MAP/QUESTION_CONTENT/SCENARIO_FOLLOWUP
  4 常量改为小程序题序(由新参考程序提取);头注重写。
- tools/migrate_sim_to_mp_order.py:45 教师模拟数据按自对合 M 重贴题号标签
  (只改标签、不改数值)→ 模拟数据_45位教师_mp题序/;原目录保留。
- advisor_norms.js:重生成,Q 键改 mp 题号,version→2026-07-15-45sim-mporder。
- advisor_ref_output:新参考程序在重贴标签数据上重生成。
- gsyg_selectFinal/index.js:删 MP_TO_PY/PY_TO_MP,buildAdvisorInput 用 mpNum,
  mpQ 恒等;verify_cf_pipeline 映射改恒等。
- 三份对拍对新参考 45/45·0 diff;新增 verify_migration_equivalence.js:
  旧链路 vs 新链路 43/45 一致,2 位(sim_009/043)因 R/P/G 同值并列的题号
  tie-break 断法不同而不同——采用新程序 tie-break 的预期结果,非缺陷。
- sync_cf 已同步云函数副本;CLAUDE.md 记录迁移全景与行为差异。

部署:重传 gsyg_selectFinal(normsVersion 变化触发老 session 自动重算一次)。
</commit_message>
<xml_diff>
--- a/tools/advisor_ref_output/AI访谈材料.xlsx
+++ b/tools/advisor_ref_output/AI访谈材料.xlsx
@@ -117,12 +117,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q3</t>
+          <t xml:space="preserve">Q6</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -177,7 +177,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -204,12 +204,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -264,7 +264,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -291,12 +291,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -351,7 +351,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -465,12 +465,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2</t>
+          <t xml:space="preserve">Q4</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -525,7 +525,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -552,12 +552,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -639,12 +639,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -699,7 +699,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -813,12 +813,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2</t>
+          <t xml:space="preserve">Q4</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -873,7 +873,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
@@ -900,12 +900,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
@@ -987,12 +987,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2</t>
+          <t xml:space="preserve">Q4</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
@@ -1074,12 +1074,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
@@ -1161,12 +1161,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1248,12 +1248,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q8</t>
+          <t xml:space="preserve">Q10</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可追问：你当时主要依据什么来排列这些做法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可追问：你当时主要依据什么来排列这些做法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -1335,12 +1335,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1395,7 +1395,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -1422,12 +1422,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2</t>
+          <t xml:space="preserve">Q4</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -1509,12 +1509,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
@@ -1596,12 +1596,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可追问：你当时主要依据什么来排列这些做法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可追问：你当时主要依据什么来排列这些做法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -1683,12 +1683,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q6</t>
+          <t xml:space="preserve">Q3</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -1857,12 +1857,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q3</t>
+          <t xml:space="preserve">Q6</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -1944,12 +1944,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2004,7 +2004,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
@@ -2205,67 +2205,67 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q3</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">飞行棋各走各的</t>
+          <t xml:space="preserve">区域停留短</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t xml:space="preserve">大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。</t>
+          <t xml:space="preserve">小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t xml:space="preserve">耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导。</t>
+          <t xml:space="preserve">提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享。</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t xml:space="preserve">暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题。</t>
+          <t xml:space="preserve">游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友。</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t xml:space="preserve">拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏。</t>
+          <t xml:space="preserve">仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因。</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t xml:space="preserve">待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。</t>
+          <t xml:space="preserve">以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t xml:space="preserve">C</t>
+          <t xml:space="preserve">D</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t xml:space="preserve">B/D</t>
+          <t xml:space="preserve">A/B</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t xml:space="preserve">教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏。</t>
+          <t xml:space="preserve">教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t xml:space="preserve">教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题。；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。</t>
+          <t xml:space="preserve">教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享。；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友。</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
@@ -2292,67 +2292,67 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q6</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">区域停留短</t>
+          <t xml:space="preserve">飞行棋各走各的</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t xml:space="preserve">小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。</t>
+          <t xml:space="preserve">大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t xml:space="preserve">提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享。</t>
+          <t xml:space="preserve">耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导。</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t xml:space="preserve">游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友。</t>
+          <t xml:space="preserve">暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题。</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t xml:space="preserve">仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因。</t>
+          <t xml:space="preserve">拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏。</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t xml:space="preserve">以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。</t>
+          <t xml:space="preserve">待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t xml:space="preserve">D</t>
+          <t xml:space="preserve">C</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t xml:space="preserve">A/B</t>
+          <t xml:space="preserve">B/D</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t xml:space="preserve">教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。</t>
+          <t xml:space="preserve">教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏。</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t xml:space="preserve">教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享。；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友。</t>
+          <t xml:space="preserve">教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题。；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
@@ -2379,42 +2379,42 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q8</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">跳绳秩序混乱</t>
+          <t xml:space="preserve">艾莎公主不运动</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t xml:space="preserve">周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。</t>
+          <t xml:space="preserve">小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t xml:space="preserve">请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏。</t>
+          <t xml:space="preserve">询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动。</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t xml:space="preserve">请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则。</t>
+          <t xml:space="preserve">提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏。</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t xml:space="preserve">提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏。</t>
+          <t xml:space="preserve">利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动。</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t xml:space="preserve">暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。</t>
+          <t xml:space="preserve">肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
@@ -2424,22 +2424,22 @@
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t xml:space="preserve">B/C</t>
+          <t xml:space="preserve">A/C</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t xml:space="preserve">教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则。</t>
+          <t xml:space="preserve">教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏。</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t xml:space="preserve">教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则。；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏。</t>
+          <t xml:space="preserve">教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动。；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动。</t>
         </is>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -2466,12 +2466,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -2526,7 +2526,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -2553,12 +2553,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -2613,7 +2613,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -2640,12 +2640,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q8</t>
+          <t xml:space="preserve">Q10</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -2700,7 +2700,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -2727,12 +2727,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q3</t>
+          <t xml:space="preserve">Q6</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -2787,7 +2787,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
@@ -2901,12 +2901,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2961,7 +2961,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
@@ -2988,12 +2988,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -3048,7 +3048,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
@@ -3075,12 +3075,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2</t>
+          <t xml:space="preserve">Q4</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -3135,7 +3135,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
@@ -3162,12 +3162,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -3222,7 +3222,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
@@ -3249,12 +3249,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -3309,7 +3309,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
@@ -3336,12 +3336,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q6</t>
+          <t xml:space="preserve">Q3</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -3396,7 +3396,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
@@ -3423,12 +3423,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
@@ -3510,12 +3510,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2</t>
+          <t xml:space="preserve">Q4</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
@@ -3597,12 +3597,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr">
@@ -3684,12 +3684,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -3744,7 +3744,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr">
@@ -3771,12 +3771,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q6</t>
+          <t xml:space="preserve">Q3</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -3831,7 +3831,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr">
@@ -3858,12 +3858,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -3918,7 +3918,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr">
@@ -4119,12 +4119,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2</t>
+          <t xml:space="preserve">Q4</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -4179,7 +4179,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr">
@@ -4293,12 +4293,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -4353,7 +4353,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可追问：你当时主要依据什么来排列这些做法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可追问：你当时主要依据什么来排列这些做法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr">
@@ -4380,12 +4380,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -4440,7 +4440,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr">
@@ -4467,12 +4467,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr">
@@ -4554,12 +4554,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr">
@@ -4641,12 +4641,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2</t>
+          <t xml:space="preserve">Q4</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -4701,7 +4701,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr">
@@ -4728,12 +4728,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q3</t>
+          <t xml:space="preserve">Q6</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -4788,7 +4788,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr">
@@ -4815,12 +4815,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -4875,7 +4875,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr">
@@ -4989,12 +4989,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q8</t>
+          <t xml:space="preserve">Q10</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -5049,7 +5049,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr">
@@ -5076,12 +5076,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q6</t>
+          <t xml:space="preserve">Q3</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr">
@@ -5163,12 +5163,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -5223,7 +5223,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr">
@@ -5250,12 +5250,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -5310,7 +5310,7 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr">
@@ -5337,12 +5337,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2</t>
+          <t xml:space="preserve">Q4</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -5397,7 +5397,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr">
@@ -5424,12 +5424,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q8</t>
+          <t xml:space="preserve">Q10</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -5484,7 +5484,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
@@ -5598,12 +5598,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q8</t>
+          <t xml:space="preserve">Q10</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr">
@@ -5685,12 +5685,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q3</t>
+          <t xml:space="preserve">Q6</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr">
@@ -5772,12 +5772,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5832,7 +5832,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr">
@@ -5859,12 +5859,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q3</t>
+          <t xml:space="preserve">Q6</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5919,7 +5919,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr">
@@ -5946,12 +5946,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q8</t>
+          <t xml:space="preserve">Q10</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -6006,7 +6006,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
@@ -6033,12 +6033,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -6093,7 +6093,7 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
@@ -6120,12 +6120,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr">
@@ -6207,12 +6207,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q3</t>
+          <t xml:space="preserve">Q6</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -6267,7 +6267,7 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr">
@@ -6294,12 +6294,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -6354,7 +6354,7 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr">
@@ -6381,12 +6381,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q6</t>
+          <t xml:space="preserve">Q3</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -6441,7 +6441,7 @@
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr">
@@ -6468,12 +6468,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -6528,7 +6528,7 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr">
@@ -6555,12 +6555,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2</t>
+          <t xml:space="preserve">Q4</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -6615,7 +6615,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr">
@@ -6642,12 +6642,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -6702,7 +6702,7 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -6903,12 +6903,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -6963,7 +6963,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
@@ -6990,12 +6990,12 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q8</t>
+          <t xml:space="preserve">Q10</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -7050,7 +7050,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -7077,12 +7077,12 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q3</t>
+          <t xml:space="preserve">Q6</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -7137,7 +7137,7 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -7164,12 +7164,12 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -7224,7 +7224,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -7425,12 +7425,12 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2</t>
+          <t xml:space="preserve">Q4</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -7485,7 +7485,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">
@@ -7512,12 +7512,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -7572,7 +7572,7 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
@@ -7686,12 +7686,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -7746,7 +7746,7 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr">
@@ -7860,12 +7860,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q3</t>
+          <t xml:space="preserve">Q6</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q91" t="inlineStr">
@@ -7947,12 +7947,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q6</t>
+          <t xml:space="preserve">Q3</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -8007,7 +8007,7 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q92" t="inlineStr">
@@ -8034,12 +8034,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -8094,7 +8094,7 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q93" t="inlineStr">
@@ -8121,12 +8121,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr">
@@ -8208,12 +8208,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -8268,7 +8268,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr">
@@ -8295,12 +8295,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -8355,7 +8355,7 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q96" t="inlineStr">
@@ -8382,12 +8382,12 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q8</t>
+          <t xml:space="preserve">Q10</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -8442,7 +8442,7 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q97" t="inlineStr">
@@ -8469,12 +8469,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -8529,7 +8529,7 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q98" t="inlineStr">
@@ -8643,12 +8643,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -8703,7 +8703,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
@@ -8730,12 +8730,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -8790,7 +8790,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">
@@ -8817,12 +8817,12 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q6</t>
+          <t xml:space="preserve">Q3</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -8877,7 +8877,7 @@
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr">
@@ -9078,12 +9078,12 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q6</t>
+          <t xml:space="preserve">Q3</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -9138,7 +9138,7 @@
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr">
@@ -9165,12 +9165,12 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -9225,7 +9225,7 @@
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr">
@@ -9426,12 +9426,12 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -9486,7 +9486,7 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr">
@@ -9513,12 +9513,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q6</t>
+          <t xml:space="preserve">Q3</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -9573,7 +9573,7 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr">
@@ -9600,12 +9600,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q8</t>
+          <t xml:space="preserve">Q10</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
@@ -9660,7 +9660,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr">
@@ -9687,12 +9687,12 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -9747,7 +9747,7 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr">
@@ -9774,12 +9774,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q7</t>
+          <t xml:space="preserve">Q9</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t xml:space="preserve">7</t>
+          <t xml:space="preserve">9</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -9834,7 +9834,7 @@
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：大班区域游戏中，轩轩和小宇一起玩飞行棋，他们将棋子摆好后，各自拿了一个骰子开始投，小宇说：“该我走。”轩轩说：“明明该我走！”相持不下，于是两人各拿一个骰子，自顾自地走自己的棋。当时提供的做法包括：教师A：耐心讲解共同游戏的规则，再以“棋手”身份加入游戏进行示范引导；教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏；教师D：待幼儿体验一轮各走各的游戏后，询问幼儿的游戏体验，提示共同游戏规则的作用。可以先从这个情境本身追问：两个孩子各走各的棋时，你当时更关注共同游戏规则的建立，还是先让他们体验这种玩法会带来什么问题？；你觉得教师怎样帮助幼儿从各玩各的，过渡到真正的共同游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，继续观察游戏进展，待区域小结时请幼儿分享游戏中的体验和问题；教师C：拿走一个骰子，请幼儿商量只有一个骰子的共同游戏规则，达成一致后再开始游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q113" t="inlineStr">
@@ -9861,12 +9861,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -9921,7 +9921,7 @@
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr">
@@ -9948,12 +9948,12 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q8</t>
+          <t xml:space="preserve">Q10</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -10008,7 +10008,7 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q115" t="inlineStr">
@@ -10035,12 +10035,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -10095,7 +10095,7 @@
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q116" t="inlineStr">
@@ -10209,12 +10209,12 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q8</t>
+          <t xml:space="preserve">Q10</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -10269,7 +10269,7 @@
       </c>
       <c r="P118" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q118" t="inlineStr">
@@ -10296,12 +10296,12 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -10356,7 +10356,7 @@
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q119" t="inlineStr">
@@ -10383,12 +10383,12 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -10443,7 +10443,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr">
@@ -10557,12 +10557,12 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -10617,7 +10617,7 @@
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q122" t="inlineStr">
@@ -10644,12 +10644,12 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q9</t>
+          <t xml:space="preserve">Q7</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -10704,7 +10704,7 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第9题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第7题这个情境。当时的情境是：小班的一次户外运动，有几个女孩子从一开始就没有选择任何体育活动项目，而是聚在一起坐在地上玩“艾莎公主”的游戏，比一比谁的鞋子最漂亮，谁的魔法最厉害。当时提供的做法包括：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏；教师C：利用艾莎公主的鞋子设计走、跑、跳等活动，并以参与者的身份邀请幼儿一起参与运动；教师D：肯定幼儿自主游戏的行为，言语引导幼儿穿着“漂亮的鞋子”参与运动。可以先从这个情境本身追问：几个女孩在户外运动时间玩艾莎公主时，你当时更关注运动目标，还是关注她们正在生成的角色游戏兴趣？；如果要把艾莎公主游戏和运动活动连接起来，你觉得教师可以怎样做才不显得生硬？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：询问幼儿没有参与运动的原因，提供丰富的活动材料吸引幼儿参与运动活动；教师B：提醒幼儿现在是运动时间，请他们等自由游戏时间再一起玩“艾莎公主”的游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q123" t="inlineStr">
@@ -10731,12 +10731,12 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q8</t>
+          <t xml:space="preserve">Q10</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t xml:space="preserve">8</t>
+          <t xml:space="preserve">10</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -10791,7 +10791,7 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：周三下午，大五班的幼儿正自发进行跳绳游戏。李老师观察后发现，挤在一起跳绳的幼儿人数较多，整个场面十分混乱，幼儿很容易出现碰撞现象。此外，由于当“柱子”的幼儿很久才能轮上跳绳，因此也显得很不耐烦。当时提供的做法包括：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师B：请幼儿说一说跳绳活动中存在的问题，并邀请幼儿一起设置跳绳的规则；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏；教师D：暂不介入，活动分享时通过照片或视频回放引导幼儿发现问题并商议解决办法。可以先从这个情境本身追问：跳绳现场混乱且可能碰撞时，你当时更倾向于立即组织秩序，还是先让幼儿自己发现问题？；在安全风险和幼儿自主制定规则之间，你觉得教师应该怎样把握介入时机？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：请幼儿暂停游戏，将幼儿分成多个小组并引导他们以小组为单位分区域开展游戏；教师C：提供更多数量和不同种类的跳绳，并言语引导幼儿分组分区同时进行跳绳游戏？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q124" t="inlineStr">
@@ -10818,12 +10818,12 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -10878,7 +10878,7 @@
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr">
@@ -10905,12 +10905,12 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -10965,7 +10965,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可追问：你当时主要依据什么来排列这些做法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可追问：你当时主要依据什么来排列这些做法？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr">
@@ -10992,12 +10992,12 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q2</t>
+          <t xml:space="preserve">Q4</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t xml:space="preserve">2</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -11052,7 +11052,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：大班建构活动中，睿睿和其他幼儿计划一起搭积木大桥，他们讨论了搭建方法，并进入区域开始搭建。就在其他幼儿在认真搭建时，睿睿发现了一块长条木板，他一会儿在地上推着走，一会儿当枪使，没有再参与小组的搭建。当时提供的做法包括：教师A：继续观察，后续分享中支持睿睿思考如何把长条木板融入小组的建构中；教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩；教师D：看到睿睿玩得开心，暂不介入，等下一次活动时再提醒他根据计划开展游戏。可以先从这个情境本身追问：睿睿离开了原来的搭桥计划去玩长条木板，你当时怎样理解他的行为：是偏离共同任务，还是出现了新的游戏线索？；面对共同建构计划和幼儿临时兴趣之间的变化，你觉得教师什么时候应该介入，什么时候可以继续观察？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：肯定睿睿的创造性玩法，询问他长条板能否当桥面，引导他参与到搭桥任务中；教师C：引导睿睿回顾计划，建议他先完成共同任务，长条木板可以等自由游戏时再玩？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr">
@@ -11079,67 +11079,67 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q3</t>
+          <t xml:space="preserve">Q2</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t xml:space="preserve">材料选择无层次</t>
+          <t xml:space="preserve">频繁求助</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t xml:space="preserve">大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。</t>
+          <t xml:space="preserve">中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t xml:space="preserve">调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡。</t>
+          <t xml:space="preserve">鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力。</t>
         </is>
       </c>
       <c r="I128" t="inlineStr">
         <is>
-          <t xml:space="preserve">暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累。</t>
+          <t xml:space="preserve">先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建。</t>
         </is>
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t xml:space="preserve">调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战。</t>
+          <t xml:space="preserve">在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤。</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t xml:space="preserve">和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。</t>
+          <t xml:space="preserve">帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。</t>
         </is>
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t xml:space="preserve">A</t>
+          <t xml:space="preserve">B</t>
         </is>
       </c>
       <c r="M128" t="inlineStr">
         <is>
-          <t xml:space="preserve">B/C</t>
+          <t xml:space="preserve">B/D</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
         <is>
-          <t xml:space="preserve">教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡。</t>
+          <t xml:space="preserve">教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建。</t>
         </is>
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t xml:space="preserve">教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累。；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战。</t>
+          <t xml:space="preserve">教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建。；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。</t>
         </is>
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第2题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr">
@@ -11166,67 +11166,67 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q4</t>
+          <t xml:space="preserve">Q6</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t xml:space="preserve">4</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t xml:space="preserve">频繁求助</t>
+          <t xml:space="preserve">材料选择无层次</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t xml:space="preserve">中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。</t>
+          <t xml:space="preserve">大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t xml:space="preserve">鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力。</t>
+          <t xml:space="preserve">调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡。</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
         <is>
-          <t xml:space="preserve">先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建。</t>
+          <t xml:space="preserve">暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累。</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
         <is>
-          <t xml:space="preserve">在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤。</t>
+          <t xml:space="preserve">调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战。</t>
         </is>
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t xml:space="preserve">帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。</t>
+          <t xml:space="preserve">和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。</t>
         </is>
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t xml:space="preserve">B</t>
+          <t xml:space="preserve">A</t>
         </is>
       </c>
       <c r="M129" t="inlineStr">
         <is>
-          <t xml:space="preserve">B/D</t>
+          <t xml:space="preserve">B/C</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
         <is>
-          <t xml:space="preserve">教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建。</t>
+          <t xml:space="preserve">教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡。</t>
         </is>
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t xml:space="preserve">教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建。；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。</t>
+          <t xml:space="preserve">教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累。；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战。</t>
         </is>
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第4题这个情境。当时的情境是：中班区域活动时，小明选择了建构区。玩了一会儿，他跑到老师面前说“老师，我不会搭……帮帮我吧”，教师问他需要什么帮助时，他一边说我不会搭，一边却很快地将房子从一层积木加高到了两层。看小明专注搭建后，老师就离开建构区了。可是没一会，小明又找了老师好几次，说“老师，帮帮我吧，我不会搭”。当时提供的做法包括：教师A：鼓励小明独立搭建，引导他思考接下来如何搭建，及时表扬他的努力；教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师C：在旁观察小明的搭建过程，并适时反馈，帮助他理清搭建步骤；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现。可以先从这个情境本身追问：小明一边说不会搭，一边又能继续加高房子，你当时怎样判断他真正需要的帮助是什么？；面对幼儿反复求助，你觉得教师怎样支持，既不替代幼儿完成，又能帮助他继续推进游戏？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：先示范搭建关键部分，请小明观察方法，再鼓励他照着继续搭建；教师D：帮小明回顾已搭建完成的部分，指导他设定小目标，尝试自己实现？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr">
@@ -11340,12 +11340,12 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q3</t>
+          <t xml:space="preserve">Q6</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -11400,7 +11400,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr">
@@ -11427,12 +11427,12 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -11487,7 +11487,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr">
@@ -11601,12 +11601,12 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q10</t>
+          <t xml:space="preserve">Q8</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -11661,7 +11661,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第10题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第8题这个情境。当时的情境是：中班上学期，幼儿在“引水游戏”中遇到了难题——水无法被引到竹片管道上。他们不断调整竹片拼接的方式，却始终没能成功，即竹片一头高于出水管道，阻碍了引流。渐渐地幼儿的探索兴趣也减弱了，有的开始玩水，有的甚至离开了水池。当时提供的做法包括：教师A：示范正确的引水方法，请幼儿注意观察并说说引水的要领，再自己试一试；教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试；教师D：投放更多辅助引水的材料，重新激起幼儿的探索兴趣，继续观察游戏进展。可以先从这个情境本身追问：孩子们引水失败、兴趣减弱时，你当时更倾向于直接示范方法，还是继续支持他们自己发现水流受阻的原因？；你觉得教师怎样提供支架，既能帮助问题解决，又保留幼儿继续探究的空间？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：加入幼儿的探索，引导他们观察水流受阻的位置，一起尝试调整竹片的摆放方式；教师C：组织幼儿就游戏困难进行讨论，寻找解决问题的方案，引导幼儿再次尝试？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr">
@@ -11688,12 +11688,12 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q6</t>
+          <t xml:space="preserve">Q3</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t xml:space="preserve">6</t>
+          <t xml:space="preserve">3</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -11748,7 +11748,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：小班幼儿瑶瑶在区域活动时，一会儿在娃娃家切切菜，一会儿到美工区搓搓橡皮泥，一会儿又开心地跑到其它区域游戏，在任何一个区域停留时间都不超过三分钟。当时提供的做法包括：教师A：提议瑶瑶完成某项游戏任务，如在娃娃家做菜，请他活动小结时分享；教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因；教师D：以同伴的身份陪伴瑶瑶在某一区域游戏，待他专注游戏后再离开。可以先从这个情境本身追问：瑶瑶在多个区域快速转换时，你当时会先把它看作注意力不集中、规则问题，还是一种探索不同材料的方式？；如果你在现场，你会先观察哪些信息来判断是否需要介入？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：游戏前提醒区域活动规则，活动结束后表扬区域游戏规则遵守得好的小朋友；教师C：仔细观察瑶瑶在不同区域的游戏情况，分析他发生迅速转移的原因？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr">
@@ -11775,12 +11775,12 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q3</t>
+          <t xml:space="preserve">Q6</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">6</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -11835,7 +11835,7 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t xml:space="preserve">请回忆第3题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
+          <t xml:space="preserve">请回忆第6题这个情境。当时的情境是：大班上学期，张老师在建构区投放了按图搭建的游戏材料，并提供了不同星级难度的任务卡供幼儿选择，但有的幼儿一上来就选择高难度的三星级任务卡，结果不能顺利完成任务；而有的幼儿始终选择低难度的一星级任务卡。这天，浩浩又连续选择了几张一星级任务卡，很快就完成了任务。当时提供的做法包括：教师A：调整任务卡提供方式，在游戏开始前根据幼儿的能力水平有针对性地发放任务卡；教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战；教师D：和浩浩回顾已完成的任务，比较不同星级的难度，邀请他选择稍有挑战的任务。可以先从这个情境本身追问：浩浩反复选择一星任务卡时，你当时更想尊重他的自主选择，还是推动他尝试更有挑战的任务？；你觉得教师应该怎样判断幼儿是需要安全感、缺少挑战意识，还是任务卡呈现方式本身需要调整？。然后可围绕其作答过程中的重点比较追问：你当时是怎样比较以下两种做法的：教师B：暂不介入，尊重幼儿的自主选择和游戏体验，只要完成任务就是一种经验积累；教师C：调整任务卡呈现方式，如增加“我想挑战”等提示，鼓励幼儿选择不同星级的挑战？如果教师提到调整过顺序，再追问：是什么信息或想法让你改变了当时的排序？请只围绕情境理解、判断依据和选项比较提问，不要提及任何内部计算指标、得分、排名、入选原因或评价性判断。</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr">

</xml_diff>